<commit_message>
test: Update transposed flow cell test to verify kinetics matching
Adds "Single cycle kinetics 1 Solution" column to the report point
table test data so kinetics lookup keys match, verifying that ka, kd,
KD, and Rmax appear in the output.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/parsers/cytiva_biacore_insight/testdata/Biacore_Insight_Transposed_FlowCells.xlsx
+++ b/tests/parsers/cytiva_biacore_insight/testdata/Biacore_Insight_Transposed_FlowCells.xlsx
@@ -425,7 +425,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -516,7 +515,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -548,7 +546,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -737,7 +734,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -887,7 +883,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -1015,8 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -1084,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1094,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1201,6 +1193,11 @@
           <t>Capture 1 Control type</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Single cycle kinetics 1 Solution</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1284,6 +1281,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1367,6 +1369,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1450,6 +1457,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1533,6 +1545,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2280,6 +2297,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2363,6 +2385,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2446,6 +2473,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2529,6 +2561,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3276,6 +3313,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3359,6 +3401,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3442,6 +3489,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3523,6 +3575,11 @@
       <c r="U31" t="inlineStr">
         <is>
           <t>Not a control</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4268,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: Recognize Evaluation-Kinetics sheet and SCK analyte lookup (#1204)
## Summary
- Accept both `"Evaluation - Kinetics"` and `"Evaluation-Kinetics"`
sheet names when loading kinetics data (some exports omit spaces around
the dash)
- For Single Cycle Kinetics (SCK) experiments, prefer `"Single cycle
kinetics 1 Solution"` over `"Analyte 1 Solution"` when building the
kinetics lookup key — otherwise ka, kd, KD, and Rmax are silently
dropped because the keys never match

## Test plan
- [x] Verified customer file now outputs all kinetics fields (ka, kd,
KD, Rmax)
- [x] All 5 existing Biacore Insight tests pass (no regressions)
- [x] All 15 Biacore discovery tests pass
- [x] Lint + mypy clean

🤖 Generated with [Claude Code](https://claude.com/claude-code)

---------

Co-authored-by: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/parsers/cytiva_biacore_insight/testdata/Biacore_Insight_Transposed_FlowCells.xlsx
+++ b/tests/parsers/cytiva_biacore_insight/testdata/Biacore_Insight_Transposed_FlowCells.xlsx
@@ -425,7 +425,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -516,7 +515,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -548,7 +546,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -737,7 +734,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -887,7 +883,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -1015,8 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -1084,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1094,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1201,6 +1193,11 @@
           <t>Capture 1 Control type</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Single cycle kinetics 1 Solution</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1284,6 +1281,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1367,6 +1369,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1450,6 +1457,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1533,6 +1545,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2280,6 +2297,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2363,6 +2385,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2446,6 +2473,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2529,6 +2561,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3276,6 +3313,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3359,6 +3401,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3442,6 +3489,11 @@
           <t>Not a control</t>
         </is>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3523,6 +3575,11 @@
       <c r="U31" t="inlineStr">
         <is>
           <t>Not a control</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>TestAnalyte</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4268,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>